<commit_message>
human label validation of embedding model
</commit_message>
<xml_diff>
--- a/src/validation/embedding_model_validation/labelling_sheet.xlsx
+++ b/src/validation/embedding_model_validation/labelling_sheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Danie\Desktop\Git Projects\DSA4264_Project\src\validation\embedding_model_validation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdama\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192A806B-EFC0-4856-BFE0-9A3638566C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB942450-63D5-45ED-9FC4-17EA1EC0F86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9220" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="1" r:id="rId1"/>
@@ -979,158 +979,158 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>25</v>
       </c>
@@ -1143,7 +1143,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1159,7 +1159,7 @@
     <col min="12" max="12" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>26</v>
       </c>
@@ -1197,7 +1197,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>0.64090000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>0.55310000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>0.44479999999999997</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1342,12 +1342,14 @@
       <c r="J5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K5" s="6"/>
+      <c r="K5" s="6">
+        <v>0</v>
+      </c>
       <c r="L5" s="5">
         <v>0.38129999999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1378,12 +1380,14 @@
       <c r="J6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K6" s="6"/>
+      <c r="K6" s="6">
+        <v>1</v>
+      </c>
       <c r="L6" s="5">
         <v>0.60670000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1414,12 +1418,14 @@
       <c r="J7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="6"/>
+      <c r="K7" s="6">
+        <v>1</v>
+      </c>
       <c r="L7" s="5">
         <v>0.51419999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -1450,12 +1456,14 @@
       <c r="J8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K8" s="6"/>
+      <c r="K8" s="6">
+        <v>0</v>
+      </c>
       <c r="L8" s="5">
         <v>0.42549999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -1486,12 +1494,14 @@
       <c r="J9" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K9" s="6"/>
+      <c r="K9" s="6">
+        <v>0</v>
+      </c>
       <c r="L9" s="5">
         <v>0.37859999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -1522,12 +1532,14 @@
       <c r="J10" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K10" s="6"/>
+      <c r="K10" s="6">
+        <v>1</v>
+      </c>
       <c r="L10" s="5">
         <v>0.57889999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -1558,12 +1570,14 @@
       <c r="J11" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K11" s="6"/>
+      <c r="K11" s="6">
+        <v>0</v>
+      </c>
       <c r="L11" s="5">
         <v>0.55110000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -1594,12 +1608,14 @@
       <c r="J12" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K12" s="6"/>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
       <c r="L12" s="5">
         <v>0.48039999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -1630,12 +1646,14 @@
       <c r="J13" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K13" s="6"/>
+      <c r="K13" s="6">
+        <v>0</v>
+      </c>
       <c r="L13" s="5">
         <v>0.40749999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="153" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -1666,12 +1684,14 @@
       <c r="J14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K14" s="6"/>
+      <c r="K14" s="6">
+        <v>2</v>
+      </c>
       <c r="L14" s="5">
         <v>0.63580000000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="153" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -1702,12 +1722,14 @@
       <c r="J15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K15" s="6"/>
+      <c r="K15" s="6">
+        <v>0</v>
+      </c>
       <c r="L15" s="5">
         <v>0.57489999999999997</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="153" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -1738,12 +1760,14 @@
       <c r="J16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="6"/>
+      <c r="K16" s="6">
+        <v>0</v>
+      </c>
       <c r="L16" s="5">
         <v>0.48980000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="153" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -1774,12 +1798,14 @@
       <c r="J17" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K17" s="6"/>
+      <c r="K17" s="6">
+        <v>0</v>
+      </c>
       <c r="L17" s="5">
         <v>0.43809999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="382.5" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -1810,12 +1836,14 @@
       <c r="J18" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K18" s="6"/>
+      <c r="K18" s="6">
+        <v>2</v>
+      </c>
       <c r="L18" s="5">
         <v>0.50270000000000004</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="382.5" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -1846,12 +1874,14 @@
       <c r="J19" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K19" s="6"/>
+      <c r="K19" s="6">
+        <v>1</v>
+      </c>
       <c r="L19" s="5">
         <v>0.49490000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="382.5" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -1882,12 +1912,14 @@
       <c r="J20" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K20" s="6"/>
+      <c r="K20" s="6">
+        <v>0</v>
+      </c>
       <c r="L20" s="5">
         <v>0.44619999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="396" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="382.5" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -1918,12 +1950,14 @@
       <c r="J21" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K21" s="6"/>
+      <c r="K21" s="6">
+        <v>0</v>
+      </c>
       <c r="L21" s="5">
         <v>0.3805</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="408" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -1954,12 +1988,14 @@
       <c r="J22" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K22" s="6"/>
+      <c r="K22" s="6">
+        <v>2</v>
+      </c>
       <c r="L22" s="5">
         <v>0.60370000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="408" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -1990,12 +2026,14 @@
       <c r="J23" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="6"/>
+      <c r="K23" s="6">
+        <v>0</v>
+      </c>
       <c r="L23" s="5">
         <v>0.57730000000000004</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="408" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -2026,12 +2064,14 @@
       <c r="J24" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K24" s="6"/>
+      <c r="K24" s="6">
+        <v>0</v>
+      </c>
       <c r="L24" s="5">
         <v>0.49740000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="408" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -2062,12 +2102,14 @@
       <c r="J25" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K25" s="6"/>
+      <c r="K25" s="6">
+        <v>0</v>
+      </c>
       <c r="L25" s="5">
         <v>0.41339999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -2098,12 +2140,14 @@
       <c r="J26" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K26" s="6"/>
+      <c r="K26" s="6">
+        <v>2</v>
+      </c>
       <c r="L26" s="5">
         <v>0.61919999999999997</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -2134,12 +2178,14 @@
       <c r="J27" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K27" s="6"/>
+      <c r="K27" s="6">
+        <v>0</v>
+      </c>
       <c r="L27" s="5">
         <v>0.59730000000000005</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -2170,12 +2216,14 @@
       <c r="J28" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K28" s="6"/>
+      <c r="K28" s="6">
+        <v>0</v>
+      </c>
       <c r="L28" s="5">
         <v>0.44929999999999998</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -2206,12 +2254,14 @@
       <c r="J29" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K29" s="6"/>
+      <c r="K29" s="6">
+        <v>0</v>
+      </c>
       <c r="L29" s="5">
         <v>0.39439999999999997</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="153" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -2242,12 +2292,14 @@
       <c r="J30" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K30" s="6"/>
+      <c r="K30" s="6">
+        <v>2</v>
+      </c>
       <c r="L30" s="5">
         <v>0.62749999999999995</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="145.19999999999999" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="140.25" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -2278,12 +2330,14 @@
       <c r="J31" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K31" s="6"/>
+      <c r="K31" s="6">
+        <v>0</v>
+      </c>
       <c r="L31" s="5">
         <v>0.55159999999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="132" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -2314,12 +2368,14 @@
       <c r="J32" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K32" s="6"/>
+      <c r="K32" s="6">
+        <v>0</v>
+      </c>
       <c r="L32" s="5">
         <v>0.45950000000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -2350,12 +2406,14 @@
       <c r="J33" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K33" s="6"/>
+      <c r="K33" s="6">
+        <v>0</v>
+      </c>
       <c r="L33" s="5">
         <v>0.4078</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="369.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -2386,12 +2444,14 @@
       <c r="J34" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K34" s="6"/>
+      <c r="K34" s="6">
+        <v>2</v>
+      </c>
       <c r="L34" s="5">
         <v>0.63500000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="369.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -2422,12 +2482,14 @@
       <c r="J35" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K35" s="6"/>
+      <c r="K35" s="6">
+        <v>1</v>
+      </c>
       <c r="L35" s="5">
         <v>0.5464</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="369.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -2458,12 +2520,14 @@
       <c r="J36" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K36" s="6"/>
+      <c r="K36" s="6">
+        <v>0</v>
+      </c>
       <c r="L36" s="5">
         <v>0.45019999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="369.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" ht="369.75" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -2494,12 +2558,14 @@
       <c r="J37" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K37" s="6"/>
+      <c r="K37" s="6">
+        <v>0</v>
+      </c>
       <c r="L37" s="5">
         <v>0.4052</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="409.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -2530,12 +2596,14 @@
       <c r="J38" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K38" s="6"/>
+      <c r="K38" s="6">
+        <v>2</v>
+      </c>
       <c r="L38" s="5">
         <v>0.56110000000000004</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="409.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -2566,12 +2634,14 @@
       <c r="J39" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K39" s="6"/>
+      <c r="K39" s="6">
+        <v>1</v>
+      </c>
       <c r="L39" s="5">
         <v>0.54479999999999995</v>
       </c>
     </row>
-    <row r="40" spans="1:12" ht="409.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -2602,12 +2672,14 @@
       <c r="J40" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K40" s="6"/>
+      <c r="K40" s="6">
+        <v>0</v>
+      </c>
       <c r="L40" s="5">
         <v>0.44750000000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="409.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" ht="395.25" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>40</v>
       </c>
@@ -2638,12 +2710,14 @@
       <c r="J41" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K41" s="6"/>
+      <c r="K41" s="6">
+        <v>0</v>
+      </c>
       <c r="L41" s="5">
         <v>0.3836</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -2674,12 +2748,14 @@
       <c r="J42" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K42" s="6"/>
+      <c r="K42" s="6">
+        <v>2</v>
+      </c>
       <c r="L42" s="5">
         <v>0.56740000000000002</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>42</v>
       </c>
@@ -2710,12 +2786,14 @@
       <c r="J43" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K43" s="6"/>
+      <c r="K43" s="6">
+        <v>1</v>
+      </c>
       <c r="L43" s="5">
         <v>0.53900000000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -2746,12 +2824,14 @@
       <c r="J44" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K44" s="6"/>
+      <c r="K44" s="6">
+        <v>1</v>
+      </c>
       <c r="L44" s="5">
         <v>0.48159999999999997</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="356.4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" ht="344.25" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
         <v>44</v>
       </c>
@@ -2782,12 +2862,14 @@
       <c r="J45" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K45" s="6"/>
+      <c r="K45" s="6">
+        <v>0</v>
+      </c>
       <c r="L45" s="5">
         <v>0.4516</v>
       </c>
     </row>
-    <row r="46" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
         <v>45</v>
       </c>
@@ -2818,12 +2900,14 @@
       <c r="J46" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="K46" s="6"/>
+      <c r="K46" s="6">
+        <v>2</v>
+      </c>
       <c r="L46" s="5">
         <v>0.56730000000000003</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
         <v>46</v>
       </c>
@@ -2854,12 +2938,14 @@
       <c r="J47" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="K47" s="6"/>
+      <c r="K47" s="6">
+        <v>1</v>
+      </c>
       <c r="L47" s="5">
         <v>0.51800000000000002</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
         <v>47</v>
       </c>
@@ -2890,12 +2976,14 @@
       <c r="J48" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K48" s="6"/>
+      <c r="K48" s="6">
+        <v>2</v>
+      </c>
       <c r="L48" s="5">
         <v>0.46560000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
         <v>48</v>
       </c>
@@ -2926,7 +3014,9 @@
       <c r="J49" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K49" s="6"/>
+      <c r="K49" s="6">
+        <v>0</v>
+      </c>
       <c r="L49" s="5">
         <v>0.39119999999999999</v>
       </c>

</xml_diff>